<commit_message>
docs(rendusrncp): add cont-03 support test evidence, sync bloc 2/4 with new support address
</commit_message>
<xml_diff>
--- a/rendusrncp/cahier_recettes.xlsx
+++ b/rendusrncp/cahier_recettes.xlsx
@@ -872,7 +872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L111"/>
+  <dimension ref="A1:L112"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="28.42578125" defaultRowHeight="23.25"/>
   <cols>
     <col width="7.28515625" customWidth="1" style="32" min="1" max="1"/>
@@ -5195,320 +5195,379 @@
     <row r="83" ht="75" customHeight="1">
       <c r="B83" s="34" t="inlineStr">
         <is>
+          <t>CONT-03</t>
+        </is>
+      </c>
+      <c r="C83" s="35" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+      <c r="D83" s="35" t="inlineStr">
+        <is>
+          <t>Fonctionnel</t>
+        </is>
+      </c>
+      <c r="E83" s="36" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="F83" s="35" t="inlineStr">
+        <is>
+          <t>Validation manuelle du canal support en conditions réelles</t>
+        </is>
+      </c>
+      <c r="G83" s="35" t="inlineStr">
+        <is>
+          <t>Formulaire /contact accessible en production, adresse support configurée (support@gauthierfitness.fr)</t>
+        </is>
+      </c>
+      <c r="H83" s="35" t="inlineStr">
+        <is>
+          <t>1. Un testeur externe soumet un message réel via /contact sur gauthierfitness.fr
+2. Le candidat consulte le message reçu sur la boîte support
+3. Le candidat répond au testeur</t>
+        </is>
+      </c>
+      <c r="I83" s="35" t="inlineStr">
+        <is>
+          <t>Le message arrive dans la boîte support configurée, avec Reply-To pointant vers l'expéditeur réel. La réponse du candidat parvient bien au testeur.</t>
+        </is>
+      </c>
+      <c r="J83" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K83" s="35" t="inlineStr">
+        <is>
+          <t>Manuel — testé le 09/07/2026 (2 itérations)</t>
+        </is>
+      </c>
+      <c r="L83" s="35" t="inlineStr">
+        <is>
+          <t>Testeur externe : Guillaume F. Question réelle sur le poids de la veste coupe-vent (produit hommes-vestes-veste-coupe-vent-900). 1re itération via gauthierfitness.help@gmail.com, réponse en 25 min. 2e itération après migration vers support@gauthierfitness.fr (OVH Email Pro), réponse en ~20 min avec signature pro complète. Preuves : preuves_recettes/contact-support-question-produit-recue.png et contact-support-question-produit-reponse.png. Alimente Bloc 4, C4.3.3 (collaboration support).</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="75" customHeight="1">
+      <c r="B84" s="34" t="inlineStr">
+        <is>
           <t>SEC-01</t>
         </is>
       </c>
-      <c r="C83" s="35" t="inlineStr">
+      <c r="C84" s="35" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="D83" s="35" t="inlineStr">
+      <c r="D84" s="35" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="E83" s="36" t="inlineStr">
+      <c r="E84" s="36" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="F83" s="35" t="inlineStr">
+      <c r="F84" s="35" t="inlineStr">
         <is>
           <t>Header HSTS présent sur prod HTTPS</t>
         </is>
       </c>
-      <c r="G83" s="35" t="inlineStr">
+      <c r="G84" s="35" t="inlineStr">
         <is>
           <t>Site servi en HTTPS via Nginx</t>
         </is>
       </c>
-      <c r="H83" s="35" t="inlineStr">
+      <c r="H84" s="35" t="inlineStr">
         <is>
           <t>1. curl -I https://gauthierfitness.fr | grep -i strict</t>
         </is>
       </c>
-      <c r="I83" s="35" t="inlineStr">
+      <c r="I84" s="35" t="inlineStr">
         <is>
           <t>Header Strict-Transport-Security retourné avec max-age et includeSubDomains.</t>
         </is>
       </c>
-      <c r="J83" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K83" s="35" t="inlineStr">
+      <c r="J84" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K84" s="35" t="inlineStr">
         <is>
           <t>Manuel curl</t>
         </is>
       </c>
-      <c r="L83" s="35" t="inlineStr">
+      <c r="L84" s="35" t="inlineStr">
         <is>
           <t>Correctif (infra/nginx/prod.conf + staging.conf, commits 6db4d70/15a5853) déployé et vérifié en direct le 08/07/2026 : curl -I sur https://gauthierfitness.fr et https://staging.gauthierfitness.fr renvoient Strict-Transport-Security: max-age=31536000; includeSubDomains. Le commentaire précédent ("non commité, non déployé") était obsolète. Capture : preuves_recettes/sec01-sec02-headers-hsts-csp-prod.png.</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="75" customHeight="1">
-      <c r="B84" s="38" t="inlineStr">
+    <row r="85" ht="75" customHeight="1">
+      <c r="B85" s="38" t="inlineStr">
         <is>
           <t>SEC-02</t>
         </is>
       </c>
-      <c r="C84" s="39" t="inlineStr">
+      <c r="C85" s="39" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="D84" s="39" t="inlineStr">
+      <c r="D85" s="39" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="E84" s="39" t="inlineStr">
+      <c r="E85" s="39" t="inlineStr">
         <is>
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F84" s="39" t="inlineStr">
+      <c r="F85" s="39" t="inlineStr">
         <is>
           <t>CSP empêche scripts inline non autorisés</t>
         </is>
       </c>
-      <c r="G84" s="39" t="inlineStr">
+      <c r="G85" s="39" t="inlineStr">
         <is>
           <t>Prod en HTTPS</t>
         </is>
       </c>
-      <c r="H84" s="39" t="inlineStr">
+      <c r="H85" s="39" t="inlineStr">
         <is>
           <t>1. Inspecter Content-Security-Policy retourné</t>
         </is>
       </c>
-      <c r="I84" s="39" t="inlineStr">
+      <c r="I85" s="39" t="inlineStr">
         <is>
           <t>CSP présent autorisant uniquement self + js.stripe.com.</t>
         </is>
       </c>
-      <c r="J84" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K84" s="39" t="inlineStr">
+      <c r="J85" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K85" s="39" t="inlineStr">
         <is>
           <t>Manuel curl</t>
         </is>
       </c>
-      <c r="L84" s="39" t="inlineStr">
+      <c r="L85" s="39" t="inlineStr">
         <is>
           <t>Correctif déployé et vérifié en direct le 08/07/2026 : curl -I sur prod et staging renvoient un header Content-Security-Policy restrictif (self + js.stripe.com + Sentry). Même correctif que SEC-01, même commit. Capture : preuves_recettes/sec01-sec02-headers-hsts-csp-prod.png.</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="75" customHeight="1">
-      <c r="B85" s="34" t="inlineStr">
+    <row r="86" ht="75" customHeight="1">
+      <c r="B86" s="34" t="inlineStr">
         <is>
           <t>SEC-03</t>
         </is>
       </c>
-      <c r="C85" s="35" t="inlineStr">
+      <c r="C86" s="35" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="D85" s="35" t="inlineStr">
+      <c r="D86" s="35" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="E85" s="36" t="inlineStr">
+      <c r="E86" s="36" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="F85" s="35" t="inlineStr">
+      <c r="F86" s="35" t="inlineStr">
         <is>
           <t>Audit composer sans vulnérabilité critique</t>
         </is>
       </c>
-      <c r="G85" s="35" t="inlineStr">
+      <c r="G86" s="35" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H85" s="35" t="inlineStr">
+      <c r="H86" s="35" t="inlineStr">
         <is>
           <t>1. composer audit (sur backend)</t>
         </is>
       </c>
-      <c r="I85" s="35" t="inlineStr">
+      <c r="I86" s="35" t="inlineStr">
         <is>
           <t>Aucune vulnérabilité critique ou high.</t>
         </is>
       </c>
-      <c r="J85" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K85" s="35" t="inlineStr">
+      <c r="J86" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K86" s="35" t="inlineStr">
         <is>
           <t>Manuel composer audit</t>
         </is>
       </c>
-      <c r="L85" s="35" t="inlineStr">
+      <c r="L86" s="35" t="inlineStr">
         <is>
           <t>composer audit exécuté le 06/07/2026 sur backend — aucune vulnérabilité.</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="75" customHeight="1">
-      <c r="B86" s="38" t="inlineStr">
+    <row r="87" ht="75" customHeight="1">
+      <c r="B87" s="38" t="inlineStr">
         <is>
           <t>SEC-04</t>
         </is>
       </c>
-      <c r="C86" s="39" t="inlineStr">
+      <c r="C87" s="39" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="D86" s="39" t="inlineStr">
+      <c r="D87" s="39" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="E86" s="36" t="inlineStr">
+      <c r="E87" s="36" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="F86" s="39" t="inlineStr">
+      <c r="F87" s="39" t="inlineStr">
         <is>
           <t>Audit npm sans vulnérabilité critique</t>
         </is>
       </c>
-      <c r="G86" s="39" t="inlineStr">
+      <c r="G87" s="39" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H86" s="39" t="inlineStr">
+      <c r="H87" s="39" t="inlineStr">
         <is>
           <t>1. npm audit (sur frontend)</t>
         </is>
       </c>
-      <c r="I86" s="39" t="inlineStr">
+      <c r="I87" s="39" t="inlineStr">
         <is>
           <t>Aucune vulnérabilité critique ou high.</t>
         </is>
       </c>
-      <c r="J86" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K86" s="39" t="inlineStr">
+      <c r="J87" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K87" s="39" t="inlineStr">
         <is>
           <t>Manuel npm audit</t>
         </is>
       </c>
-      <c r="L86" s="39" t="inlineStr">
+      <c r="L87" s="39" t="inlineStr">
         <is>
           <t>npm audit exécuté le 06/07/2026 sur frontend — aucune vulnérabilité.</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="75" customHeight="1">
-      <c r="B87" s="34" t="inlineStr">
+    <row r="88" ht="75" customHeight="1">
+      <c r="B88" s="34" t="inlineStr">
         <is>
           <t>SEC-05</t>
         </is>
       </c>
-      <c r="C87" s="35" t="inlineStr">
+      <c r="C88" s="35" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="D87" s="35" t="inlineStr">
+      <c r="D88" s="35" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="E87" s="36" t="inlineStr">
+      <c r="E88" s="36" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="F87" s="35" t="inlineStr">
+      <c r="F88" s="35" t="inlineStr">
         <is>
           <t>MySQL non exposé depuis Internet</t>
         </is>
       </c>
-      <c r="G87" s="35" t="inlineStr">
+      <c r="G88" s="35" t="inlineStr">
         <is>
           <t>VPS prod</t>
         </is>
       </c>
-      <c r="H87" s="35" t="inlineStr">
+      <c r="H88" s="35" t="inlineStr">
         <is>
           <t>1. nmap -p 3306 &lt;ip_vps_prod&gt;</t>
         </is>
       </c>
-      <c r="I87" s="35" t="inlineStr">
+      <c r="I88" s="35" t="inlineStr">
         <is>
           <t>Port 3306 filtré ou fermé (jamais ouvert).</t>
         </is>
       </c>
-      <c r="J87" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K87" s="35" t="inlineStr">
+      <c r="J88" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K88" s="35" t="inlineStr">
         <is>
           <t>Manuel nmap</t>
         </is>
       </c>
-      <c r="L87" s="35" t="inlineStr">
+      <c r="L88" s="35" t="inlineStr">
         <is>
           <t>Test de connexion TCP externe sur le port 3306 le 06/07/2026 — fermé sur prod (51.38.234.197) et staging (51.210.15.118).</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="75" customHeight="1">
-      <c r="B88" s="38" t="inlineStr">
+    <row r="89" ht="75" customHeight="1">
+      <c r="B89" s="38" t="inlineStr">
         <is>
           <t>A11Y-01</t>
         </is>
       </c>
-      <c r="C88" s="39" t="inlineStr">
+      <c r="C89" s="39" t="inlineStr">
         <is>
           <t>Accessibilité</t>
         </is>
       </c>
-      <c r="D88" s="39" t="inlineStr">
+      <c r="D89" s="39" t="inlineStr">
         <is>
           <t>Accessibilité</t>
         </is>
       </c>
-      <c r="E88" s="39" t="inlineStr">
+      <c r="E89" s="39" t="inlineStr">
         <is>
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F88" s="39" t="inlineStr">
+      <c r="F89" s="39" t="inlineStr">
         <is>
           <t>Navigation clavier sur le parcours d'achat</t>
         </is>
       </c>
-      <c r="G88" s="39" t="inlineStr">
+      <c r="G89" s="39" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H88" s="39" t="inlineStr">
+      <c r="H89" s="39" t="inlineStr">
         <is>
           <t>1. Home → Tab → focus sur premier item de nav
 2. Continuer Tab → traverser Header, Hero, catalogue
@@ -5516,967 +5575,950 @@
 4. Ajouter au panier via Espace/Entrée</t>
         </is>
       </c>
-      <c r="I88" s="39" t="inlineStr">
+      <c r="I89" s="39" t="inlineStr">
         <is>
           <t>Tous les éléments interactifs sont accessibles au clavier. Focus visible. Ordre logique.</t>
         </is>
       </c>
-      <c r="J88" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K88" s="39" t="inlineStr">
+      <c r="J89" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K89" s="39" t="inlineStr">
         <is>
           <t>Manuel</t>
         </is>
       </c>
-      <c r="L88" s="39" t="inlineStr">
+      <c r="L89" s="39" t="inlineStr">
         <is>
           <t>Testé le 06/07/2026 sur staging (parcours Home → catalogue → fiche produit → ajout panier, entièrement au clavier). Focus visible à chaque étape, ordre logique respecté. Preuve : capture vidéo de l'écran + captures d'écran (à joindre dans preuves_recettes/).</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="75" customHeight="1">
-      <c r="B89" s="34" t="inlineStr">
+    <row r="90" ht="75" customHeight="1">
+      <c r="B90" s="34" t="inlineStr">
         <is>
           <t>A11Y-02</t>
         </is>
       </c>
-      <c r="C89" s="35" t="inlineStr">
+      <c r="C90" s="35" t="inlineStr">
         <is>
           <t>Accessibilité</t>
         </is>
       </c>
-      <c r="D89" s="35" t="inlineStr">
+      <c r="D90" s="35" t="inlineStr">
         <is>
           <t>Accessibilité</t>
         </is>
       </c>
-      <c r="E89" s="35" t="inlineStr">
+      <c r="E90" s="35" t="inlineStr">
         <is>
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F89" s="35" t="inlineStr">
+      <c r="F90" s="35" t="inlineStr">
         <is>
           <t>Score Lighthouse Accessibility ≥ 90 sur Home</t>
         </is>
       </c>
-      <c r="G89" s="35" t="inlineStr">
+      <c r="G90" s="35" t="inlineStr">
         <is>
           <t>Build prod servi</t>
         </is>
       </c>
-      <c r="H89" s="35" t="inlineStr">
+      <c r="H90" s="35" t="inlineStr">
         <is>
           <t>1. Chrome DevTools → Lighthouse → Accessibility</t>
         </is>
       </c>
-      <c r="I89" s="35" t="inlineStr">
+      <c r="I90" s="35" t="inlineStr">
         <is>
           <t>Score ≥ 90.</t>
         </is>
       </c>
-      <c r="J89" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K89" s="35" t="inlineStr">
+      <c r="J90" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K90" s="35" t="inlineStr">
         <is>
           <t>Manuel Lighthouse</t>
         </is>
       </c>
-      <c r="L89" s="35" t="inlineStr">
+      <c r="L90" s="35" t="inlineStr">
         <is>
           <t>Audit Lighthouse Home après correctifs (RNCP-Lighthouse-GF29, 05/07/2026) — score Accessibility 100 (≥ 90 requis).</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="75" customHeight="1">
-      <c r="B90" s="38" t="inlineStr">
+    <row r="91" ht="75" customHeight="1">
+      <c r="B91" s="38" t="inlineStr">
         <is>
           <t>A11Y-03</t>
         </is>
       </c>
-      <c r="C90" s="39" t="inlineStr">
+      <c r="C91" s="39" t="inlineStr">
         <is>
           <t>Accessibilité</t>
         </is>
       </c>
-      <c r="D90" s="39" t="inlineStr">
+      <c r="D91" s="39" t="inlineStr">
         <is>
           <t>Accessibilité</t>
         </is>
       </c>
-      <c r="E90" s="39" t="inlineStr">
+      <c r="E91" s="39" t="inlineStr">
         <is>
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F90" s="39" t="inlineStr">
+      <c r="F91" s="39" t="inlineStr">
         <is>
           <t>Alt présent sur toutes les images de produit</t>
         </is>
       </c>
-      <c r="G90" s="39" t="inlineStr">
+      <c r="G91" s="39" t="inlineStr">
         <is>
           <t>Page catalogue chargée</t>
         </is>
       </c>
-      <c r="H90" s="39" t="inlineStr">
+      <c r="H91" s="39" t="inlineStr">
         <is>
           <t>1. Inspecter DOM, vérifier &lt;img alt="..."&gt;</t>
         </is>
       </c>
-      <c r="I90" s="39" t="inlineStr">
+      <c r="I91" s="39" t="inlineStr">
         <is>
           <t>Chaque image produit a un alt non vide. Images décoratives ont alt="".</t>
         </is>
       </c>
-      <c r="J90" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K90" s="39" t="inlineStr">
+      <c r="J91" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K91" s="39" t="inlineStr">
         <is>
           <t>Manuel inspecteur</t>
         </is>
       </c>
-      <c r="L90" s="39" t="inlineStr">
+      <c r="L91" s="39" t="inlineStr">
         <is>
           <t>Audit Lighthouse Home après correctifs — audit « image-alt » à 100 %. Vérifié sur Home uniquement ; produit/panier/checkout restent à vérifier si besoin.</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="75" customHeight="1">
-      <c r="B91" s="34" t="inlineStr">
+    <row r="92" ht="75" customHeight="1">
+      <c r="B92" s="34" t="inlineStr">
         <is>
           <t>UI-01</t>
         </is>
       </c>
-      <c r="C91" s="35" t="inlineStr">
+      <c r="C92" s="35" t="inlineStr">
         <is>
           <t>Frontend UI</t>
         </is>
       </c>
-      <c r="D91" s="35" t="inlineStr">
+      <c r="D92" s="35" t="inlineStr">
         <is>
           <t>Structurel</t>
         </is>
       </c>
-      <c r="E91" s="35" t="inlineStr">
+      <c r="E92" s="35" t="inlineStr">
         <is>
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F91" s="35" t="inlineStr">
+      <c r="F92" s="35" t="inlineStr">
         <is>
           <t>axios intercepteur attache Bearer token</t>
         </is>
       </c>
-      <c r="G91" s="35" t="inlineStr">
+      <c r="G92" s="35" t="inlineStr">
         <is>
           <t>Token en localStorage</t>
         </is>
       </c>
-      <c r="H91" s="35" t="inlineStr">
+      <c r="H92" s="35" t="inlineStr">
         <is>
           <t>1. Appeler n'importe quel endpoint</t>
         </is>
       </c>
-      <c r="I91" s="35" t="inlineStr">
+      <c r="I92" s="35" t="inlineStr">
         <is>
           <t>Header Authorization: Bearer &lt;token&gt; ajouté à chaque requête.</t>
         </is>
       </c>
-      <c r="J91" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K91" s="35" t="inlineStr">
+      <c r="J92" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K92" s="35" t="inlineStr">
         <is>
           <t>Jest axios.test.js::attaches Bearer token</t>
         </is>
       </c>
-      <c r="L91" s="35" t="inlineStr">
-        <is>
-          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="75" customHeight="1">
-      <c r="B92" s="38" t="inlineStr">
+      <c r="L92" s="35" t="inlineStr">
+        <is>
+          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="75" customHeight="1">
+      <c r="B93" s="38" t="inlineStr">
         <is>
           <t>UI-02</t>
         </is>
       </c>
-      <c r="C92" s="39" t="inlineStr">
+      <c r="C93" s="39" t="inlineStr">
         <is>
           <t>Frontend UI</t>
         </is>
       </c>
-      <c r="D92" s="39" t="inlineStr">
+      <c r="D93" s="39" t="inlineStr">
         <is>
           <t>Structurel</t>
         </is>
       </c>
-      <c r="E92" s="39" t="inlineStr">
+      <c r="E93" s="39" t="inlineStr">
         <is>
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F92" s="39" t="inlineStr">
+      <c r="F93" s="39" t="inlineStr">
         <is>
           <t>axios 401 purge le token automatiquement</t>
         </is>
       </c>
-      <c r="G92" s="39" t="inlineStr">
+      <c r="G93" s="39" t="inlineStr">
         <is>
           <t>Token expired en localStorage</t>
         </is>
       </c>
-      <c r="H92" s="39" t="inlineStr">
+      <c r="H93" s="39" t="inlineStr">
         <is>
           <t>1. Endpoint renvoie 401</t>
         </is>
       </c>
-      <c r="I92" s="39" t="inlineStr">
+      <c r="I93" s="39" t="inlineStr">
         <is>
           <t>localStorage.token supprimé. User doit re-login.</t>
         </is>
       </c>
-      <c r="J92" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K92" s="39" t="inlineStr">
+      <c r="J93" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K93" s="39" t="inlineStr">
         <is>
           <t>Jest axios.test.js::removes token from localStorage on 401</t>
         </is>
       </c>
-      <c r="L92" s="39" t="inlineStr">
-        <is>
-          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="75" customHeight="1">
-      <c r="B93" s="34" t="inlineStr">
+      <c r="L93" s="39" t="inlineStr">
+        <is>
+          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="46.5" customHeight="1">
+      <c r="B94" s="34" t="inlineStr">
         <is>
           <t>UI-03</t>
         </is>
       </c>
-      <c r="C93" s="35" t="inlineStr">
+      <c r="C94" s="35" t="inlineStr">
         <is>
           <t>Frontend UI</t>
         </is>
       </c>
-      <c r="D93" s="35" t="inlineStr">
+      <c r="D94" s="35" t="inlineStr">
         <is>
           <t>Fonctionnel</t>
         </is>
       </c>
-      <c r="E93" s="36" t="inlineStr">
+      <c r="E94" s="36" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="F93" s="35" t="inlineStr">
+      <c r="F94" s="35" t="inlineStr">
         <is>
           <t>AuthProvider login persiste user + token</t>
         </is>
       </c>
-      <c r="G93" s="35" t="inlineStr">
+      <c r="G94" s="35" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H93" s="35" t="inlineStr">
+      <c r="H94" s="35" t="inlineStr">
         <is>
           <t>1. login("alice@a.fr", "secret")
 2. Inspecter localStorage</t>
         </is>
       </c>
-      <c r="I93" s="35" t="inlineStr">
+      <c r="I94" s="35" t="inlineStr">
         <is>
           <t>token + user (JSON) en localStorage. Context expose isAuthenticated=true.</t>
         </is>
       </c>
-      <c r="J93" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K93" s="35" t="inlineStr">
+      <c r="J94" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K94" s="35" t="inlineStr">
         <is>
           <t>Jest auth.test.jsx::login stores token + user</t>
         </is>
       </c>
-      <c r="L93" s="35" t="inlineStr">
-        <is>
-          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="46.5" customHeight="1">
-      <c r="B94" s="38" t="inlineStr">
+      <c r="L94" s="35" t="inlineStr">
+        <is>
+          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="46.5" customHeight="1">
+      <c r="B95" s="38" t="inlineStr">
         <is>
           <t>UI-04</t>
         </is>
       </c>
-      <c r="C94" s="39" t="inlineStr">
+      <c r="C95" s="39" t="inlineStr">
         <is>
           <t>Frontend UI</t>
         </is>
       </c>
-      <c r="D94" s="39" t="inlineStr">
+      <c r="D95" s="39" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="E94" s="36" t="inlineStr">
+      <c r="E95" s="36" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="F94" s="39" t="inlineStr">
+      <c r="F95" s="39" t="inlineStr">
         <is>
           <t>AuthProvider 401 sur /me → purge tout</t>
         </is>
       </c>
-      <c r="G94" s="39" t="inlineStr">
+      <c r="G95" s="39" t="inlineStr">
         <is>
           <t>Token expired</t>
         </is>
       </c>
-      <c r="H94" s="39" t="inlineStr">
+      <c r="H95" s="39" t="inlineStr">
         <is>
           <t>1. Bootstrap au mount, /me renvoie 401</t>
         </is>
       </c>
-      <c r="I94" s="39" t="inlineStr">
+      <c r="I95" s="39" t="inlineStr">
         <is>
           <t>Token + user purgés du localStorage. isAuthenticated=false.</t>
         </is>
       </c>
-      <c r="J94" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K94" s="39" t="inlineStr">
+      <c r="J95" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K95" s="39" t="inlineStr">
         <is>
           <t>Jest auth.test.jsx::bootstrap clears token on /me returning 401</t>
         </is>
       </c>
-      <c r="L94" s="39" t="inlineStr">
-        <is>
-          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="46.5" customHeight="1">
-      <c r="B95" s="34" t="inlineStr">
+      <c r="L95" s="39" t="inlineStr">
+        <is>
+          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" s="34" t="inlineStr">
         <is>
           <t>UI-05</t>
         </is>
       </c>
-      <c r="C95" s="35" t="inlineStr">
+      <c r="C96" s="35" t="inlineStr">
         <is>
           <t>Frontend UI</t>
         </is>
       </c>
-      <c r="D95" s="35" t="inlineStr">
+      <c r="D96" s="35" t="inlineStr">
         <is>
           <t>Fonctionnel</t>
         </is>
       </c>
-      <c r="E95" s="35" t="inlineStr">
+      <c r="E96" s="35" t="inlineStr">
         <is>
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F95" s="35" t="inlineStr">
+      <c r="F96" s="35" t="inlineStr">
         <is>
           <t>AuthProvider 500 ne purge pas (backend down)</t>
         </is>
       </c>
-      <c r="G95" s="35" t="inlineStr">
+      <c r="G96" s="35" t="inlineStr">
         <is>
           <t>Token valide, backend down</t>
         </is>
       </c>
-      <c r="H95" s="35" t="inlineStr">
+      <c r="H96" s="35" t="inlineStr">
         <is>
           <t>1. Bootstrap, /me renvoie 500</t>
         </is>
       </c>
-      <c r="I95" s="35" t="inlineStr">
+      <c r="I96" s="35" t="inlineStr">
         <is>
           <t>Token + user CONSERVÉS. User reste connecté visuellement.</t>
         </is>
       </c>
-      <c r="J95" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K95" s="35" t="inlineStr">
+      <c r="J96" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K96" s="35" t="inlineStr">
         <is>
           <t>Jest auth.test.jsx::bootstrap keeps token when /me errors with 500</t>
         </is>
       </c>
-      <c r="L95" s="35" t="inlineStr">
-        <is>
-          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="B96" s="38" t="inlineStr">
+      <c r="L96" s="35" t="inlineStr">
+        <is>
+          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="46.5" customHeight="1">
+      <c r="B97" s="38" t="inlineStr">
         <is>
           <t>UI-06</t>
         </is>
       </c>
-      <c r="C96" s="39" t="inlineStr">
+      <c r="C97" s="39" t="inlineStr">
         <is>
           <t>Frontend UI</t>
         </is>
       </c>
-      <c r="D96" s="39" t="inlineStr">
+      <c r="D97" s="39" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="E96" s="36" t="inlineStr">
+      <c r="E97" s="36" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="F96" s="39" t="inlineStr">
+      <c r="F97" s="39" t="inlineStr">
         <is>
           <t>ProtectedRoute redirige /login si pas auth</t>
         </is>
       </c>
-      <c r="G96" s="39" t="inlineStr">
+      <c r="G97" s="39" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H96" s="39" t="inlineStr">
+      <c r="H97" s="39" t="inlineStr">
         <is>
           <t>1. Naviguer /dashboard sans token</t>
         </is>
       </c>
-      <c r="I96" s="39" t="inlineStr">
+      <c r="I97" s="39" t="inlineStr">
         <is>
           <t>Redirection vers /login.</t>
         </is>
       </c>
-      <c r="J96" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K96" s="39" t="inlineStr">
+      <c r="J97" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K97" s="39" t="inlineStr">
         <is>
           <t>Jest ProtectedRoutes.test.jsx + Cypress admin.cy.js</t>
         </is>
       </c>
-      <c r="L96" s="39" t="inlineStr">
+      <c r="L97" s="39" t="inlineStr">
         <is>
           <t>Suite Jest rejouée le 08/07/2026 : ProtectedRoute.test.jsx 3/3 vert (39 tests Jest frontend au total, tous verts). Capture : preuves_recettes/ui06-protectedroute-test.png.</t>
         </is>
       </c>
     </row>
-    <row r="97" ht="46.5" customHeight="1">
-      <c r="B97" s="34" t="inlineStr">
+    <row r="98">
+      <c r="B98" s="34" t="inlineStr">
         <is>
           <t>UI-07</t>
         </is>
       </c>
-      <c r="C97" s="35" t="inlineStr">
+      <c r="C98" s="35" t="inlineStr">
         <is>
           <t>Frontend UI</t>
         </is>
       </c>
-      <c r="D97" s="35" t="inlineStr">
+      <c r="D98" s="35" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="E97" s="36" t="inlineStr">
+      <c r="E98" s="36" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="F97" s="35" t="inlineStr">
+      <c r="F98" s="35" t="inlineStr">
         <is>
           <t>AdminRoute affiche un message d'accès refusé si connecté mais pas admin</t>
         </is>
       </c>
-      <c r="G97" s="35" t="inlineStr">
+      <c r="G98" s="35" t="inlineStr">
         <is>
           <t>User customer connecté</t>
         </is>
       </c>
-      <c r="H97" s="35" t="inlineStr">
+      <c r="H98" s="35" t="inlineStr">
         <is>
           <t>1. Naviguer /admin</t>
         </is>
       </c>
-      <c r="I97" s="35" t="inlineStr">
+      <c r="I98" s="35" t="inlineStr">
         <is>
           <t>Message "Accès refusé" affiché. Pas de redirection, pas d'affichage du panel admin.</t>
         </is>
       </c>
-      <c r="J97" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K97" s="35" t="inlineStr">
+      <c r="J98" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K98" s="35" t="inlineStr">
         <is>
           <t>Jest AdminRoutes.test.jsx::shows an access-denied message when authenticated but not admin</t>
         </is>
       </c>
-      <c r="L97" s="35" t="inlineStr">
-        <is>
-          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="B98" s="38" t="inlineStr">
+      <c r="L98" s="35" t="inlineStr">
+        <is>
+          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="63" customHeight="1">
+      <c r="B99" s="38" t="inlineStr">
         <is>
           <t>UI-08</t>
         </is>
       </c>
-      <c r="C98" s="39" t="inlineStr">
+      <c r="C99" s="39" t="inlineStr">
         <is>
           <t>Frontend UI</t>
         </is>
       </c>
-      <c r="D98" s="39" t="inlineStr">
+      <c r="D99" s="39" t="inlineStr">
         <is>
           <t>Fonctionnel</t>
         </is>
       </c>
-      <c r="E98" s="39" t="inlineStr">
+      <c r="E99" s="39" t="inlineStr">
         <is>
           <t>Basse</t>
         </is>
       </c>
-      <c r="F98" s="39" t="inlineStr">
+      <c r="F99" s="39" t="inlineStr">
         <is>
           <t>ProductCard affiche prix au format X.XX €</t>
         </is>
       </c>
-      <c r="G98" s="39" t="inlineStr">
+      <c r="G99" s="39" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H98" s="39" t="inlineStr">
+      <c r="H99" s="39" t="inlineStr">
         <is>
           <t>1. Rendre ProductCard avec price_ttc=29.9</t>
         </is>
       </c>
-      <c r="I98" s="39" t="inlineStr">
+      <c r="I99" s="39" t="inlineStr">
         <is>
           <t>Affiche "29.90 €" (2 décimales).</t>
         </is>
       </c>
-      <c r="J98" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K98" s="39" t="inlineStr">
+      <c r="J99" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K99" s="39" t="inlineStr">
         <is>
           <t>Jest ProductCard.test.jsx::renders product name and price</t>
         </is>
       </c>
-      <c r="L98" s="39" t="inlineStr">
-        <is>
-          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="63" customHeight="1">
-      <c r="B99" s="34" t="inlineStr">
+      <c r="L99" s="39" t="inlineStr">
+        <is>
+          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" s="34" t="inlineStr">
         <is>
           <t>UI-09</t>
         </is>
       </c>
-      <c r="C99" s="35" t="inlineStr">
+      <c r="C100" s="35" t="inlineStr">
         <is>
           <t>Frontend UI</t>
         </is>
       </c>
-      <c r="D99" s="35" t="inlineStr">
+      <c r="D100" s="35" t="inlineStr">
         <is>
           <t>Fonctionnel</t>
         </is>
       </c>
-      <c r="E99" s="35" t="inlineStr">
+      <c r="E100" s="35" t="inlineStr">
         <is>
           <t>Basse</t>
         </is>
       </c>
-      <c r="F99" s="35" t="inlineStr">
+      <c r="F100" s="35" t="inlineStr">
         <is>
           <t>ProductCard change d'image au hover</t>
         </is>
       </c>
-      <c r="G99" s="35" t="inlineStr">
+      <c r="G100" s="35" t="inlineStr">
         <is>
           <t>Produit avec main_image et hover_image</t>
         </is>
       </c>
-      <c r="H99" s="35" t="inlineStr">
+      <c r="H100" s="35" t="inlineStr">
         <is>
           <t>1. mouseEnter sur la carte</t>
         </is>
       </c>
-      <c r="I99" s="35" t="inlineStr">
+      <c r="I100" s="35" t="inlineStr">
         <is>
           <t>Le src de l'image passe de main_image à hover_image.</t>
         </is>
       </c>
-      <c r="J99" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K99" s="35" t="inlineStr">
+      <c r="J100" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K100" s="35" t="inlineStr">
         <is>
           <t>Jest ProductCard.test.jsx::shows hover image on mouse enter</t>
         </is>
       </c>
-      <c r="L99" s="35" t="inlineStr">
-        <is>
-          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="B100" s="38" t="inlineStr">
+      <c r="L100" s="35" t="inlineStr">
+        <is>
+          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="46.5" customHeight="1">
+      <c r="B101" s="38" t="inlineStr">
         <is>
           <t>INFRA-01</t>
         </is>
       </c>
-      <c r="C100" s="39" t="inlineStr">
+      <c r="C101" s="39" t="inlineStr">
         <is>
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="D100" s="39" t="inlineStr">
+      <c r="D101" s="39" t="inlineStr">
         <is>
           <t>Fonctionnel</t>
         </is>
       </c>
-      <c r="E100" s="36" t="inlineStr">
+      <c r="E101" s="36" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="F100" s="39" t="inlineStr">
+      <c r="F101" s="39" t="inlineStr">
         <is>
           <t>Health check /api/health renvoie 200</t>
         </is>
       </c>
-      <c r="G100" s="39" t="inlineStr">
+      <c r="G101" s="39" t="inlineStr">
         <is>
           <t>Backend démarré</t>
         </is>
       </c>
-      <c r="H100" s="39" t="inlineStr">
+      <c r="H101" s="39" t="inlineStr">
         <is>
           <t>1. GET /api/health</t>
         </is>
       </c>
-      <c r="I100" s="39" t="inlineStr">
+      <c r="I101" s="39" t="inlineStr">
         <is>
           <t>Réponse 200 {status:"ok", env:"production"}.</t>
         </is>
       </c>
-      <c r="J100" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K100" s="39" t="inlineStr">
+      <c r="J101" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K101" s="39" t="inlineStr">
         <is>
           <t>PHPUnit HealthTest</t>
         </is>
       </c>
-      <c r="L100" s="39" t="inlineStr">
-        <is>
-          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="46.5" customHeight="1">
-      <c r="B101" s="34" t="inlineStr">
+      <c r="L101" s="39" t="inlineStr">
+        <is>
+          <t>Suite complète rejouée le 06/07/2026 : 164 tests PHPUnit backend + 39 tests Jest frontend, tous verts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="46.5" customHeight="1">
+      <c r="B102" s="34" t="inlineStr">
         <is>
           <t>INFRA-02</t>
         </is>
       </c>
-      <c r="C101" s="35" t="inlineStr">
+      <c r="C102" s="35" t="inlineStr">
         <is>
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="D101" s="35" t="inlineStr">
+      <c r="D102" s="35" t="inlineStr">
         <is>
           <t>Structurel</t>
         </is>
       </c>
-      <c r="E101" s="36" t="inlineStr">
+      <c r="E102" s="36" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="F101" s="35" t="inlineStr">
+      <c r="F102" s="35" t="inlineStr">
         <is>
           <t>CI backend verte sur PR</t>
         </is>
       </c>
-      <c r="G101" s="35" t="inlineStr">
+      <c r="G102" s="35" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H101" s="35" t="inlineStr">
+      <c r="H102" s="35" t="inlineStr">
         <is>
           <t>1. Push sur GF{n}
 2. Ouvrir PR vers develop</t>
         </is>
       </c>
-      <c r="I101" s="35" t="inlineStr">
+      <c r="I102" s="35" t="inlineStr">
         <is>
           <t>Workflow CI : PHPUnit + Pint + Build image + Trigger infra → tous verts.</t>
         </is>
       </c>
-      <c r="J101" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K101" s="35" t="inlineStr">
+      <c r="J102" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K102" s="35" t="inlineStr">
         <is>
           <t>GitHub Actions backend ci-cd.yml</t>
         </is>
       </c>
-      <c r="L101" s="35" t="inlineStr">
+      <c r="L102" s="35" t="inlineStr">
         <is>
           <t>CI backend vérifiée verte le 08/07/2026 : sur push develop/main (ex. run GitHub Actions #28949610914) et sur pull request (ex. run #28868839895, PR GF31-V1GF-Ready -&gt; develop). ci-cd.yml se déclenche bien sur push ET pull_request vers main/develop. Capture : preuves_recettes/infra02-ci-backend-pr.png.</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="46.5" customHeight="1">
-      <c r="B102" s="38" t="inlineStr">
+    <row r="103" ht="69.75" customHeight="1">
+      <c r="B103" s="38" t="inlineStr">
         <is>
           <t>INFRA-03</t>
         </is>
       </c>
-      <c r="C102" s="39" t="inlineStr">
+      <c r="C103" s="39" t="inlineStr">
         <is>
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="D102" s="39" t="inlineStr">
+      <c r="D103" s="39" t="inlineStr">
         <is>
           <t>Structurel</t>
         </is>
       </c>
-      <c r="E102" s="36" t="inlineStr">
+      <c r="E103" s="36" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="F102" s="39" t="inlineStr">
+      <c r="F103" s="39" t="inlineStr">
         <is>
           <t>CI frontend verte sur PR</t>
         </is>
       </c>
-      <c r="G102" s="39" t="inlineStr">
+      <c r="G103" s="39" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H102" s="39" t="inlineStr">
+      <c r="H103" s="39" t="inlineStr">
         <is>
           <t>1. Push + PR</t>
         </is>
       </c>
-      <c r="I102" s="39" t="inlineStr">
+      <c r="I103" s="39" t="inlineStr">
         <is>
           <t>Workflow CI : ESLint + Build Vite + Jest + Build image → tous verts.</t>
         </is>
       </c>
-      <c r="J102" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K102" s="39" t="inlineStr">
+      <c r="J103" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K103" s="39" t="inlineStr">
         <is>
           <t>GitHub Actions frontend ci-cd.yml</t>
         </is>
       </c>
-      <c r="L102" s="39" t="inlineStr">
+      <c r="L103" s="39" t="inlineStr">
         <is>
           <t>CI frontend vérifiée verte le 08/07/2026 : sur push develop/main (ex. run #28925409791) et sur pull request (ex. run Dependabot #28925617135). ci-cd.yml se déclenche bien sur push ET pull_request vers main/develop. Capture : preuves_recettes/infra03-ci-frontend-pr.png.</t>
         </is>
       </c>
     </row>
-    <row r="103" ht="69.75" customHeight="1">
-      <c r="B103" s="34" t="inlineStr">
+    <row r="104" ht="46.5" customHeight="1">
+      <c r="B104" s="34" t="inlineStr">
         <is>
           <t>INFRA-04</t>
         </is>
       </c>
-      <c r="C103" s="35" t="inlineStr">
+      <c r="C104" s="35" t="inlineStr">
         <is>
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="D103" s="35" t="inlineStr">
+      <c r="D104" s="35" t="inlineStr">
         <is>
           <t>Structurel</t>
         </is>
       </c>
-      <c r="E103" s="36" t="inlineStr">
+      <c r="E104" s="36" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="F103" s="35" t="inlineStr">
+      <c r="F104" s="35" t="inlineStr">
         <is>
           <t>Pipeline complet : staging → e2e → prod</t>
         </is>
       </c>
-      <c r="G103" s="35" t="inlineStr">
+      <c r="G104" s="35" t="inlineStr">
         <is>
           <t>Push sur develop puis main</t>
         </is>
       </c>
-      <c r="H103" s="35" t="inlineStr">
+      <c r="H104" s="35" t="inlineStr">
         <is>
           <t>1. Push develop → staging auto deploy + e2e Cypress
 2. Merge dans main → trigger manuel prod</t>
         </is>
       </c>
-      <c r="I103" s="35" t="inlineStr">
+      <c r="I104" s="35" t="inlineStr">
         <is>
           <t>Staging green. E2E Cypress green. Prod deploy manuel OK avec health check 200 à la fin.</t>
         </is>
       </c>
-      <c r="J103" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K103" s="35" t="inlineStr">
+      <c r="J104" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K104" s="35" t="inlineStr">
         <is>
           <t>GitHub Actions infra deploy.yml</t>
         </is>
       </c>
-      <c r="L103" s="35" t="inlineStr">
+      <c r="L104" s="35" t="inlineStr">
         <is>
           <t>Pipeline complet vérifié le 08/07/2026 : run infra #28949784465 (staging, déclenché par repository_dispatch après CI backend/frontend) -&gt; Staging Deployment vert (48s) -&gt; Tests E2E Cypress vert (1m24s). Déploiement prod le plus récent : run #28883415233 (workflow_dispatch manuel, 07/07/2026, vert, 42s). Health check confirmé en direct le 08/07/2026 : GET https://gauthierfitness.fr/api/health -&gt; 200 {"status":"ok"}. Capture : preuves_recettes/infra04-pipeline-staging-e2e.png.</t>
         </is>
       </c>
     </row>
-    <row r="104" ht="46.5" customHeight="1">
-      <c r="B104" s="34" t="inlineStr">
+    <row r="105">
+      <c r="B105" s="34" t="inlineStr">
         <is>
           <t>INFRA-05</t>
         </is>
       </c>
-      <c r="C104" s="35" t="inlineStr">
+      <c r="C105" s="35" t="inlineStr">
         <is>
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="D104" s="35" t="inlineStr">
+      <c r="D105" s="35" t="inlineStr">
         <is>
           <t>Structurel</t>
         </is>
       </c>
-      <c r="E104" s="36" t="inlineStr">
+      <c r="E105" s="36" t="inlineStr">
         <is>
           <t>Haute</t>
         </is>
       </c>
-      <c r="F104" s="35" t="inlineStr">
+      <c r="F105" s="35" t="inlineStr">
         <is>
           <t>Pipeline complet :  production</t>
         </is>
       </c>
-      <c r="G104" s="35" t="inlineStr">
+      <c r="G105" s="35" t="inlineStr">
         <is>
           <t>Déclenchement manuel validé</t>
         </is>
       </c>
-      <c r="H104" s="35" t="inlineStr">
+      <c r="H105" s="35" t="inlineStr">
         <is>
           <t>Merge dans main → trigger manuel prod</t>
         </is>
       </c>
-      <c r="I104" s="35" t="inlineStr">
+      <c r="I105" s="35" t="inlineStr">
         <is>
           <t>Prod deploy manuel OK avec health check 200 à la fin.</t>
         </is>
       </c>
-      <c r="J104" s="37" t="inlineStr">
-        <is>
-          <t>Passé</t>
-        </is>
-      </c>
-      <c r="K104" s="35" t="inlineStr">
+      <c r="J105" s="37" t="inlineStr">
+        <is>
+          <t>Passé</t>
+        </is>
+      </c>
+      <c r="K105" s="35" t="inlineStr">
         <is>
           <t>GitHub Actions infra deploy.yml</t>
         </is>
       </c>
-      <c r="L104" s="35" t="inlineStr">
+      <c r="L105" s="35" t="inlineStr">
         <is>
           <t>Pipeline complet vérifié le 08/07/2026 : run infra #28973278625 (commit 2504e06, Production Deployment 52s, approuvé manuellement par Charles). Capture : preuves_recettes/infra05-pipeline-production.png.</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="B108" s="42" t="inlineStr">
+    <row r="109">
+      <c r="B109" s="42" t="inlineStr">
         <is>
           <t>Total scénarios : 95</t>
         </is>
       </c>
-      <c r="C108" s="43" t="n"/>
-      <c r="D108" s="44" t="n"/>
-      <c r="E108" s="41" t="n"/>
-      <c r="F108" s="41" t="n"/>
-      <c r="G108" s="41" t="n"/>
-      <c r="H108" s="41" t="n"/>
-      <c r="I108" s="41" t="n"/>
-      <c r="J108" s="41" t="n"/>
-      <c r="K108" s="41" t="n"/>
-      <c r="L108" s="41" t="n"/>
-    </row>
-    <row r="109">
-      <c r="B109" s="45" t="inlineStr">
-        <is>
-          <t>Légende statut : "À jouer" (gris) / "Passé" (vert) / "Échec" (rouge)</t>
-        </is>
-      </c>
-      <c r="C109" s="41" t="n"/>
-      <c r="D109" s="46" t="n"/>
+      <c r="C109" s="43" t="n"/>
+      <c r="D109" s="44" t="n"/>
       <c r="E109" s="41" t="n"/>
       <c r="F109" s="41" t="n"/>
       <c r="G109" s="41" t="n"/>
@@ -6489,7 +6531,7 @@
     <row r="110">
       <c r="B110" s="45" t="inlineStr">
         <is>
-          <t>Mettre à jour la colonne Statut au fil des exécutions.</t>
+          <t>Légende statut : "À jouer" (gris) / "Passé" (vert) / "Échec" (rouge)</t>
         </is>
       </c>
       <c r="C110" s="41" t="n"/>
@@ -6504,9 +6546,26 @@
       <c r="L110" s="41" t="n"/>
     </row>
     <row r="111">
-      <c r="B111" s="47" t="n"/>
-      <c r="C111" s="40" t="n"/>
-      <c r="D111" s="48" t="n"/>
+      <c r="B111" s="45" t="inlineStr">
+        <is>
+          <t>Mettre à jour la colonne Statut au fil des exécutions.</t>
+        </is>
+      </c>
+      <c r="C111" s="41" t="n"/>
+      <c r="D111" s="46" t="n"/>
+      <c r="E111" s="41" t="n"/>
+      <c r="F111" s="41" t="n"/>
+      <c r="G111" s="41" t="n"/>
+      <c r="H111" s="41" t="n"/>
+      <c r="I111" s="41" t="n"/>
+      <c r="J111" s="41" t="n"/>
+      <c r="K111" s="41" t="n"/>
+      <c r="L111" s="41" t="n"/>
+    </row>
+    <row r="112">
+      <c r="B112" s="47" t="n"/>
+      <c r="C112" s="40" t="n"/>
+      <c r="D112" s="48" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="B9:L102"/>
@@ -6542,7 +6601,6 @@
       <c r="C1" s="20" t="n"/>
       <c r="D1" s="21" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="23" t="inlineStr">
         <is>
@@ -6690,11 +6748,9 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18"/>
-    <row r="19"/>
+        <v>3</v>
+      </c>
+    </row>
     <row r="20">
       <c r="A20" s="23" t="inlineStr">
         <is>
@@ -6722,7 +6778,7 @@
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23">
@@ -6755,8 +6811,6 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="23" t="inlineStr">
         <is>
@@ -6794,7 +6848,7 @@
         </is>
       </c>
       <c r="B31" s="4" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="32">
@@ -6807,8 +6861,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33"/>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="23" t="inlineStr">
         <is>
@@ -6836,7 +6888,7 @@
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="38">
@@ -6859,7 +6911,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40"/>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="12" t="inlineStr">
         <is>
@@ -6867,7 +6918,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>